<commit_message>
Changes updated on reconcilattion agent
</commit_message>
<xml_diff>
--- a/public/Combined-Input.xlsx
+++ b/public/Combined-Input.xlsx
@@ -639,13 +639,13 @@
         <v>0</v>
       </c>
       <c r="W2" t="n">
-        <v>4354.24</v>
+        <v>4280.32</v>
       </c>
       <c r="X2" t="n">
-        <v>4354.24</v>
+        <v>4280.32</v>
       </c>
       <c r="Y2" t="n">
-        <v>4354.24</v>
+        <v>4280.32</v>
       </c>
     </row>
     <row r="3">
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>138</v>
+        <v>176</v>
       </c>
       <c r="R9" t="n">
         <v>1965</v>
@@ -1368,19 +1368,19 @@
         <v>4021.6</v>
       </c>
       <c r="U9" t="n">
-        <v>3153.3</v>
+        <v>4021.6</v>
       </c>
       <c r="V9" t="n">
-        <v>-868.3</v>
+        <v>0</v>
       </c>
       <c r="W9" t="n">
-        <v>3153.3</v>
+        <v>3952.46</v>
       </c>
       <c r="X9" t="n">
-        <v>3153.3</v>
+        <v>3952.46</v>
       </c>
       <c r="Y9" t="n">
-        <v>3153.3</v>
+        <v>3952.46</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
Changes on POC button in chatbot
</commit_message>
<xml_diff>
--- a/public/Combined-Input.xlsx
+++ b/public/Combined-Input.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>176</v>
+        <v>99</v>
       </c>
       <c r="R2" t="n">
         <v>2128</v>
@@ -633,10 +633,10 @@
         <v>4354.24</v>
       </c>
       <c r="U2" t="n">
-        <v>4354.24</v>
+        <v>2449.26</v>
       </c>
       <c r="V2" t="n">
-        <v>0</v>
+        <v>-1904.98</v>
       </c>
       <c r="W2" t="n">
         <v>4280.32</v>

</xml_diff>

<commit_message>
Expansion and minimizing the chatbot screen
</commit_message>
<xml_diff>
--- a/public/Combined-Input.xlsx
+++ b/public/Combined-Input.xlsx
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>99</v>
+        <v>176</v>
       </c>
       <c r="R2" t="n">
         <v>2128</v>
@@ -633,10 +633,10 @@
         <v>4354.24</v>
       </c>
       <c r="U2" t="n">
-        <v>2449.26</v>
+        <v>4354.24</v>
       </c>
       <c r="V2" t="n">
-        <v>-1904.98</v>
+        <v>0</v>
       </c>
       <c r="W2" t="n">
         <v>4280.32</v>

</xml_diff>